<commit_message>
Unprotect the template, and top the size bands out at 500+
The downloaded sheet could not be typed into. The input cells were technically
unlocked, but sheet protection was still on, and that blocks the things a client
actually does with a spreadsheet: pasting a block, inserting a row, sorting. The
protection existed to stop a stray paste destroying the headers, which was the
wrong way round, because the parser already tolerates a mangled sheet. It scores
rows to find the header and matches columns by name, so a broken header row
costs us nothing and a locked sheet cost the client everything.

All three tabs now carry no sheetProtection element at all, checked in the xlsx
itself rather than through openpyxl, and a value written into a data cell after
download reads back correctly.

Size bands stop at 500+ rather than splitting 500-999 from 1,000+. Above 500 the
comparator does not change enough to be worth asking.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Zigbert-Benchmarking-Template.xlsx
+++ b/public/Zigbert-Benchmarking-Template.xlsx
@@ -165,9 +165,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -185,9 +183,7 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="5" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
+    <xf numFmtId="3" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -621,7 +617,7 @@
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>0-49 / 50-99 / 100-249 / 250-499 / 500-999 / 1,000+</t>
+          <t>0-49 / 50-99 / 100-249 / 250-499 / 500+</t>
         </is>
       </c>
     </row>
@@ -751,7 +747,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="E024"/>
   <mergeCells count="7">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
@@ -4326,7 +4321,6 @@
       <c r="E505" s="6" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="E024"/>
   <mergeCells count="3">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
@@ -8403,7 +8397,6 @@
       <c r="F505" s="6" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="E024"/>
   <mergeCells count="3">
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A2:F2"/>

</xml_diff>